<commit_message>
T-1222: carry the role view through the mints, and re-derive what the withdrawals moved
</commit_message>
<xml_diff>
--- a/chicago/reference/resident-research/T-0463/T-0463_resident_research_working.xlsx
+++ b/chicago/reference/resident-research/T-0463/T-0463_resident_research_working.xlsx
@@ -2341,7 +2341,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>soap_and_candle_maker (attested)</t>
+          <t>none_recorded (reconstructed)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>dry_goods_merchant (attested)</t>
+          <t>none_recorded (reconstructed)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>dry_goods_merchant (attested)</t>
+          <t>none_recorded (reconstructed)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>grocer (attested)</t>
+          <t>none_recorded (reconstructed)</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>

</xml_diff>